<commit_message>
Fix import: 1) Parse actual date from Excel (dd/MM or dd/MM/yyyy). 2) App.tsx functional state updates. 3) Phong grid force 5 cols.
</commit_message>
<xml_diff>
--- a/dulieu_test_lich_cong_tac.xlsx
+++ b/dulieu_test_lich_cong_tac.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tải xuống\_workspace_kpi_new_full (12)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F931D4-5650-44F0-9EA3-2CC31CA74DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D404322-578D-418E-B2D2-7417AB05DF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,7 +103,7 @@
     <t>Thứ 7 (29/08)</t>
   </si>
   <si>
-    <t>Chủ nhật 30/08)</t>
+    <t>Chủ nhật (30/08)</t>
   </si>
 </sst>
 </file>
@@ -217,11 +217,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -555,7 +555,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -593,7 +593,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -631,7 +631,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -669,7 +669,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -707,7 +707,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -745,7 +745,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -783,7 +783,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="2" t="s">

</xml_diff>

<commit_message>
Fix sidebar className template literal bug. Layout: Sidebar (leaders/phong/vung1/vung2 vertical) + Matrix (shows 'Làm việc tại cơ quan') + Detail tables bottom (HIDES 'Làm việc tại cơ quan'). Matrix parses all 4 leaders from Excel.
</commit_message>
<xml_diff>
--- a/dulieu_test_lich_cong_tac.xlsx
+++ b/dulieu_test_lich_cong_tac.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tải xuống\_workspace_kpi_new_full (12)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D404322-578D-418E-B2D2-7417AB05DF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5C58D36-B799-4490-8254-60131B207D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,22 +33,6 @@
     <t>Buổi</t>
   </si>
   <si>
-    <t>Đào Trọng Truyền
-(Trưởng phòng)</t>
-  </si>
-  <si>
-    <t>Đào Thị Hiếu
-(Phó Trưởng phòng)</t>
-  </si>
-  <si>
-    <t>Vũ Tuấn Hùng
-(Phó Trưởng phòng)</t>
-  </si>
-  <si>
-    <t>Phạm Văn Tự
-(Phó Trưởng phòng)</t>
-  </si>
-  <si>
     <t>Sáng</t>
   </si>
   <si>
@@ -104,6 +88,22 @@
   </si>
   <si>
     <t>Chủ nhật (30/08)</t>
+  </si>
+  <si>
+    <t>Đào Thị Hiếu
+(Phó Trưởng Thống kê)</t>
+  </si>
+  <si>
+    <t>Vũ Tuấn Hùng
+(Phó Trưởng Thống kê)</t>
+  </si>
+  <si>
+    <t>Phạm Văn Tự
+(Phó Trưởng Thống kê)</t>
+  </si>
+  <si>
+    <t>Đào Trọng Truyến
+(Trưởng Thống kê)</t>
   </si>
 </sst>
 </file>
@@ -542,282 +542,282 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7"/>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7"/>
       <c r="B5" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7"/>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7"/>
       <c r="B11" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="7"/>
       <c r="B15" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>